<commit_message>
Update example output files from validation testing
Regenerated Excel files with latest code after setup fixes.
All examples validated and producing correct output:
- Nebraska K-12 Finance: 8.6 KB
- Radioactive Waste: 10.8 KB
- Director Networks: 9.9 KB
- Clean Air Act 1970: 14.5 KB

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/hayden_case_studies/clean_air_act_1970.xlsx
+++ b/examples/hayden_case_studies/clean_air_act_1970.xlsx
@@ -663,7 +663,7 @@
           <t>information: Referrals of Clean Air Act violations for civil and criminal...</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>rule: National Ambient Air Quality Standards for six criteria poll...
 information: Technical guidance for SIP development, emissions inventorie...
@@ -1217,17 +1217,17 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Environmental Justice Communities</t>
+          <t>Pollution Control Equipment Industry</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Industrial facilities disproportionately impact environmental justice communities through proximity and exposure patterns</t>
+          <t>Electric utilities install pollution control equipment to meet NSPS and SIP requirements</t>
         </is>
       </c>
       <c r="D2" s="10" t="n">
@@ -1237,7 +1237,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Industrial facilities emit criteria pollutants and hazardous air pollutants affecting nearby populations</t>
+          <t>Electric power plants emit SO2 and NOx causing acid rain and respiratory health impacts</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
@@ -1262,12 +1262,12 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Pollution Control Equipment Industry</t>
+          <t>Environmental Justice Communities</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Industrial facilities install control technology to comply with federal and state emissions limits</t>
+          <t>Industrial facilities disproportionately impact environmental justice communities through proximity and exposure patterns</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
@@ -1277,17 +1277,17 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Pollution Control Equipment Industry</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Industry associations lobby Congress on compliance timelines and economic impacts</t>
+          <t>Industrial facilities install control technology to comply with federal and state emissions limits</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
@@ -1297,21 +1297,21 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Industry trade groups advocate for flexible compliance timelines and cost considerations in rulemaking</t>
+          <t>Industrial facilities emit criteria pollutants and hazardous air pollutants affecting nearby populations</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1337,37 +1337,37 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Electric power plants emit SO2 and NOx causing acid rain and respiratory health impacts</t>
+          <t>Technology suppliers provide emission control equipment enabling regulatory compliance</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Air Quality Research Institutions</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Pollution Control Equipment Industry</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Electric utilities install pollution control equipment to meet NSPS and SIP requirements</t>
+          <t>Research institutions provide scientific basis for NAAQS and regulatory decisions</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
@@ -1377,37 +1377,37 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Congress grants EPA regulatory authority over air pollution through NAAQS, NSPS, NESHAPS, and mobile source standards</t>
+          <t>EPA regulates electric power plant emissions through NSPS and SIP requirements</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Congress mandates state leadership in air quality management through State Implementation Plans</t>
+          <t>EPA regulates industrial emissions through technology-based standards</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
@@ -1422,16 +1422,16 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>EPA regulates industrial emissions through technology-based standards</t>
+          <t>EPA refers significant violations to Department of Justice for enforcement actions</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>EPA refers significant violations to Department of Justice for enforcement actions</t>
+          <t>Clean Air Act implementation delivers substantial public health benefits through dramatic pollution reductions</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
@@ -1462,16 +1462,16 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>EPA regulates electric power plant emissions through NSPS and SIP requirements</t>
+          <t>EPA imposes technology-forcing emissions standards on automobile manufacturers</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1482,12 +1482,12 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>EPA imposes technology-forcing emissions standards on automobile manufacturers</t>
+          <t>EPA sets national air quality standards that states must achieve through SIPs</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
@@ -1497,17 +1497,17 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Clean Air Act implementation delivers substantial public health benefits through dramatic pollution reductions</t>
+          <t>Industry trade groups advocate for flexible compliance timelines and cost considerations in rulemaking</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
@@ -1517,37 +1517,37 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>EPA sets national air quality standards that states must achieve through SIPs</t>
+          <t>Industry associations lobby Congress on compliance timelines and economic impacts</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Automobile manufacturers forced to adopt catalytic converter technology beginning 1975 model year</t>
+          <t>CASAC provides independent scientific peer review of air quality standards since 1977</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
@@ -1562,62 +1562,62 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Automobile manufacturers emit air pollutants that impact public health, with dramatic reductions post-1975 due to catalytic converters</t>
+          <t>Automobile manufacturers forced to adopt catalytic converter technology beginning 1975 model year</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Air Quality Research Institutions</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Research institutions provide scientific basis for NAAQS and regulatory decisions</t>
+          <t>Automobile manufacturers emit air pollutants that impact public health, with dramatic reductions post-1975 due to catalytic converters</t>
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Technology suppliers provide emission control equipment enabling regulatory compliance</t>
+          <t>States submit implementation plans for EPA approval, demonstrating path to NAAQS compliance</t>
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>CASAC provides independent scientific peer review of air quality standards since 1977</t>
+          <t>Environmental organizations advocate for strong air quality protections and sue to enforce compliance</t>
         </is>
       </c>
       <c r="D22" s="10" t="n">
@@ -1657,7 +1657,7 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1667,27 +1667,27 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Environmental organizations advocate for strong air quality protections and sue to enforce compliance</t>
+          <t>Congress grants EPA regulatory authority over air pollution through NAAQS, NSPS, NESHAPS, and mobile source standards</t>
         </is>
       </c>
       <c r="D24" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
+          <t>U.S. Congress</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
           <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Environmental Protection Agency (EPA)</t>
-        </is>
-      </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>States submit implementation plans for EPA approval, demonstrating path to NAAQS compliance</t>
+          <t>Congress mandates state leadership in air quality management through State Implementation Plans</t>
         </is>
       </c>
       <c r="D25" s="10" t="n">
@@ -1769,27 +1769,31 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Environmental Justice Communities</t>
+          <t>Pollution Control Equipment Industry</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Disproportionate exposure to industrial air pollution in low-income and minority communities located near facilities</t>
+          <t>Purchase and installation of scrubbers, electrostatic precipitators, and baghouses for SO2 and particulate control</t>
         </is>
       </c>
       <c r="E2" s="11" t="n"/>
       <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H2" s="11" t="n"/>
       <c r="I2" s="11" t="n">
         <v>0.9</v>
@@ -1798,7 +1802,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1813,11 +1817,11 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Sulfur dioxide from industrial sources: 5.6 kg/km²/day (1970) reduced to 0.6 kg/km²/day by 2010</t>
+          <t>Sulfur dioxide from power plants: 9.0 kg/km²/day (1970) reduced to 3.0 kg/km²/day by 2010</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>5.6</v>
+        <v>9</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -1830,7 +1834,7 @@
         </is>
       </c>
       <c r="H3" s="11" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="I3" s="11" t="n">
         <v>0.95</v>
@@ -1839,7 +1843,7 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -1854,13 +1858,25 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Particulate matter from industry: 50% reduction by 1980 through industrial emission controls</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n"/>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="11" t="n"/>
+          <t>Nitrogen oxides from power plants: 2.5 kg/km²/day (1970) reduced to 1.5 kg/km²/day by 2010</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>kg/km²/day</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>1.5</v>
+      </c>
       <c r="I4" s="11" t="n">
         <v>0.95</v>
       </c>
@@ -1873,26 +1889,22 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Pollution Control Equipment Industry</t>
+          <t>Environmental Justice Communities</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Investment in pollution control technology to meet NSPS standards</t>
+          <t>Disproportionate exposure to industrial air pollution in low-income and minority communities located near facilities</t>
         </is>
       </c>
       <c r="E5" s="11" t="n"/>
       <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G5" s="9" t="n"/>
       <c r="H5" s="11" t="n"/>
       <c r="I5" s="11" t="n">
         <v>0.9</v>
@@ -1901,27 +1913,31 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Pollution Control Equipment Industry</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Lobbying for technology feasibility timelines and economic impact considerations in legislation</t>
+          <t>Investment in pollution control technology to meet NSPS standards</t>
         </is>
       </c>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H6" s="11" t="n"/>
       <c r="I6" s="11" t="n">
         <v>0.9</v>
@@ -1930,70 +1946,68 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Technical comments on proposed rules, compliance cost analyses, requests for deadline extensions</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="9" t="n"/>
+          <t>Sulfur dioxide from industrial sources: 5.6 kg/km²/day (1970) reduced to 0.6 kg/km²/day by 2010</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>kg/km²/day</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>continuous</t>
         </is>
       </c>
-      <c r="H7" s="11" t="n"/>
+      <c r="H7" s="11" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I7" s="11" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Civil penalties and consent decrees for violations (e.g., 2024 enforcement actions: $13M+ in penalties)</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>13000000</v>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>USD in penalties</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>event_triggered</t>
-        </is>
-      </c>
+          <t>Particulate matter from industry: 50% reduction by 1980 through industrial emission controls</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
       <c r="H8" s="11" t="n"/>
       <c r="I8" s="11" t="n">
         <v>0.95</v>
@@ -2002,40 +2016,38 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Sulfur dioxide from power plants: 9.0 kg/km²/day (1970) reduced to 3.0 kg/km²/day by 2010</t>
+          <t>Civil penalties and consent decrees for violations (e.g., 2024 enforcement actions: $13M+ in penalties)</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>9</v>
+        <v>13000000</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>kg/km²/day</t>
+          <t>USD in penalties</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>continuous</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>3</v>
-      </c>
+          <t>event_triggered</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
         <v>0.95</v>
       </c>
@@ -2043,40 +2055,28 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Nitrogen oxides from power plants: 2.5 kg/km²/day (1970) reduced to 1.5 kg/km²/day by 2010</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>kg/km²/day</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>1.5</v>
-      </c>
+          <t>Catalytic converter technology enabling 90% reduction in hydrocarbons and CO emissions</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="11" t="n"/>
       <c r="I10" s="11" t="n">
         <v>0.95</v>
       </c>
@@ -2084,22 +2084,22 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Air Quality Research Institutions</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Pollution Control Equipment Industry</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Purchase and installation of scrubbers, electrostatic precipitators, and baghouses for SO2 and particulate control</t>
+          <t>Air quality research on health effects, emissions modeling, and control technology effectiveness</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>
@@ -2117,22 +2117,22 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Legislative authority to set National Ambient Air Quality Standards (NAAQS) for six criteria pollutants</t>
+          <t>New Source Performance Standards (NSPS) for coal-fired power plants limiting SO2 and NOx emissions</t>
         </is>
       </c>
       <c r="E12" s="11" t="n"/>
@@ -2146,51 +2146,45 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Federal appropriations for EPA operations and grants to states</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>1400000000</v>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>USD/year</t>
-        </is>
-      </c>
+          <t>Continuous emissions monitoring requirements for compliance verification</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="9" t="n"/>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -2200,7 +2194,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Mandatory deadlines: NAAQS by 1971, state compliance by 1975 (later extended to 1977)</t>
+          <t>New Source Performance Standards for major industrial categories (steel, cement, chemicals)</t>
         </is>
       </c>
       <c r="E14" s="11" t="n"/>
@@ -2214,22 +2208,22 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Requirement to develop State Implementation Plans (SIPs) to achieve NAAQS</t>
+          <t>National Emission Standards for Hazardous Air Pollutants (NESHAPS)</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -2243,30 +2237,34 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Federal planning grants to state air pollution control agencies (authorized under 1967 Air Quality Act, continued)</t>
+          <t>Referrals of Clean Air Act violations for civil and criminal prosecution</t>
         </is>
       </c>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="17">
@@ -2277,17 +2275,17 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>New Source Performance Standards for major industrial categories (steel, cement, chemicals)</t>
+          <t>Dramatic air quality improvements: PM2.5 reduced to 35.1% of 1970 levels, combined six pollutants down 78% (1970-2020)</t>
         </is>
       </c>
       <c r="E17" s="11" t="n"/>
@@ -2295,7 +2293,7 @@
       <c r="G17" s="9" t="n"/>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="18">
@@ -2306,7 +2304,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -2316,7 +2314,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>National Emission Standards for Hazardous Air Pollutants (NESHAPS)</t>
+          <t>Mobile source emission standards: 90% reduction in hydrocarbons and CO by 1975, NOx by 1976</t>
         </is>
       </c>
       <c r="E18" s="11" t="n"/>
@@ -2335,29 +2333,25 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Referrals of Clean Air Act violations for civil and criminal prosecution</t>
+          <t>Certification requirements for new vehicles and warranty requirements for emission control equipment (8 years/80,000 miles)</t>
         </is>
       </c>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G19" s="9" t="n"/>
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2368,21 +2362,27 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>New Source Performance Standards (NSPS) for coal-fired power plants limiting SO2 and NOx emissions</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="9" t="n"/>
+          <t>Enforcement authority with penalties up to $45,268 per noncompliant vehicle</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>45268</v>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>USD per vehicle</t>
+        </is>
+      </c>
       <c r="G20" s="9" t="n"/>
       <c r="H20" s="11" t="n"/>
       <c r="I20" s="11" t="n">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -2407,16 +2407,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Continuous emissions monitoring requirements for compliance verification</t>
+          <t>National Ambient Air Quality Standards for six criteria pollutants (CO, lead, NO2, ozone, PM, SO2)</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="9" t="n"/>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G21" s="9" t="n"/>
       <c r="H21" s="11" t="n"/>
       <c r="I21" s="11" t="n">
         <v>1</v>
@@ -2430,17 +2426,17 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Mobile source emission standards: 90% reduction in hydrocarbons and CO by 1975, NOx by 1976</t>
+          <t>Technical guidance for SIP development, emissions inventories, and monitoring requirements</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
@@ -2448,7 +2444,7 @@
       <c r="G22" s="9" t="n"/>
       <c r="H22" s="11" t="n"/>
       <c r="I22" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="23">
@@ -2459,17 +2455,17 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Certification requirements for new vehicles and warranty requirements for emission control equipment (8 years/80,000 miles)</t>
+          <t>SIP approval authority and enforcement backstop (EPA can impose Federal Implementation Plan if state fails)</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -2483,57 +2479,55 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Enforcement authority with penalties up to $45,268 per noncompliant vehicle</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="n">
-        <v>45268</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>USD per vehicle</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="n"/>
+          <t>Technical comments on proposed rules, compliance cost analyses, requests for deadline extensions</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H24" s="11" t="n"/>
       <c r="I24" s="11" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Dramatic air quality improvements: PM2.5 reduced to 35.1% of 1970 levels, combined six pollutants down 78% (1970-2020)</t>
+          <t>Lobbying for technology feasibility timelines and economic impact considerations in legislation</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -2541,33 +2535,37 @@
       <c r="G25" s="9" t="n"/>
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>National Ambient Air Quality Standards for six criteria pollutants (CO, lead, NO2, ozone, PM, SO2)</t>
+          <t>Independent scientific review of NAAQS criteria documents and recommendations (established 1977 amendments)</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="9" t="n"/>
-      <c r="G26" s="9" t="n"/>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="11" t="n">
         <v>1</v>
@@ -2576,59 +2574,81 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Technical guidance for SIP development, emissions inventories, and monitoring requirements</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="9" t="n"/>
-      <c r="G27" s="9" t="n"/>
+          <t>Purchase of catalytic converters for all 1975+ model year vehicles at $300-1000 per unit</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>USD per vehicle</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>SIP approval authority and enforcement backstop (EPA can impose Federal Implementation Plan if state fails)</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="9" t="n"/>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="11" t="n"/>
+          <t>Nitrogen oxides from vehicles: 5.2 kg/km²/day (1970) reduced to 2.2 kg/km²/day by 2010</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>kg/km²/day</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>2.2</v>
+      </c>
       <c r="I28" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="29">
@@ -2639,102 +2659,84 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Purchase of catalytic converters for all 1975+ model year vehicles at $300-1000 per unit</t>
-        </is>
-      </c>
-      <c r="E29" s="11" t="n">
-        <v>500</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>USD per vehicle</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+          <t>Particulate matter from vehicles: &gt;90% reduction from 1970 levels due to diesel particulate filters and cleaner engines</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Nitrogen oxides from vehicles: 5.2 kg/km²/day (1970) reduced to 2.2 kg/km²/day by 2010</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>kg/km²/day</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
-      <c r="H30" s="11" t="n">
-        <v>2.2</v>
-      </c>
+          <t>State Implementation Plans detailing how state will achieve NAAQS (Utah submitted January 1972)</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Particulate matter from vehicles: &gt;90% reduction from 1970 levels due to diesel particulate filters and cleaner engines</t>
+          <t>Emissions inventories, air quality monitoring data, and compliance reports</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="11" t="n">
         <v>0.95</v>
@@ -2743,7 +2745,7 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Air Quality Research Institutions</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -2753,12 +2755,12 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Air quality research on health effects, emissions modeling, and control technology effectiveness</t>
+          <t>Advocacy for stringent NAAQS, petitions for new standards, and litigation to enforce deadlines</t>
         </is>
       </c>
       <c r="E32" s="11" t="n"/>
@@ -2770,28 +2772,28 @@
       </c>
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Catalytic converter technology enabling 90% reduction in hydrocarbons and CO emissions</t>
+          <t>Legislative advocacy for Clean Air Act passage and amendments, public health documentation</t>
         </is>
       </c>
       <c r="E33" s="11" t="n"/>
@@ -2799,13 +2801,13 @@
       <c r="G33" s="9" t="n"/>
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="11" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -2815,21 +2817,17 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Independent scientific review of NAAQS criteria documents and recommendations (established 1977 amendments)</t>
+          <t>Legislative authority to set National Ambient Air Quality Standards (NAAQS) for six criteria pollutants</t>
         </is>
       </c>
       <c r="E34" s="11" t="n"/>
       <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G34" s="9" t="n"/>
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="11" t="n">
         <v>1</v>
@@ -2838,36 +2836,46 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Legislative advocacy for Clean Air Act passage and amendments, public health documentation</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
+          <t>Federal appropriations for EPA operations and grants to states</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>1400000000</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>USD/year</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -2882,40 +2890,36 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Advocacy for stringent NAAQS, petitions for new standards, and litigation to enforce deadlines</t>
+          <t>Mandatory deadlines: NAAQS by 1971, state compliance by 1975 (later extended to 1977)</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
       <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G36" s="9" t="n"/>
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="11" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
+          <t>U.S. Congress</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
           <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>Environmental Protection Agency (EPA)</t>
-        </is>
-      </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>State Implementation Plans detailing how state will achieve NAAQS (Utah submitted January 1972)</t>
+          <t>Requirement to develop State Implementation Plans (SIPs) to achieve NAAQS</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -2929,34 +2933,30 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
+          <t>U.S. Congress</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
           <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>Environmental Protection Agency (EPA)</t>
-        </is>
-      </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Emissions inventories, air quality monitoring data, and compliance reports</t>
+          <t>Federal planning grants to state air pollution control agencies (authorized under 1967 Air Quality Act, continued)</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
       <c r="F38" s="9" t="n"/>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G38" s="9" t="n"/>
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update example outputs from fresh test run
Regenerated all 4 example demonstration XLSX files from scratch following
setup validation. All examples executed successfully with updated outputs.

Example Results:
- Nebraska K-12 Finance: 5 components, 9 deliveries (12 KB)
- Radioactive Waste Policy: 11 components, 33 deliveries (10.6 KB)
- Corporate Director Networks: 10 components, 27 deliveries (9.6 KB)
- Clean Air Act 1970: 18 components, 37 deliveries (14.2 KB)

Removed VALIDATION_SUMMARY.md as validation is complete and documented
in SETUP_FIXES.md and SETUP_GUIDE.md.

All examples demonstrate Hayden's SFM methodology with multiple deliveries
per cell, proper cell descriptions, and temporal modeling where applicable.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/hayden_case_studies/clean_air_act_1970.xlsx
+++ b/examples/hayden_case_studies/clean_air_act_1970.xlsx
@@ -47,6 +47,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
@@ -55,12 +61,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
         <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -629,7 +629,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>authority: Requirement to develop State Implementation Plans (SIPs) to ...
 money: Federal planning grants to state air pollution control agenc...</t>
@@ -658,12 +658,12 @@
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>information: Referrals of Clean Air Act violations for civil and criminal...</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>rule: National Ambient Air Quality Standards for six criteria poll...
 information: Technical guidance for SIP development, emissions inventorie...
@@ -671,20 +671,20 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>rule: Mobile source emission standards: 90% reduction in hydrocarb...
 rule: Certification requirements for new vehicles and warranty req...
 authority: Enforcement authority with penalties up to $45,268 per nonco...</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>rule: New Source Performance Standards (NSPS) for coal-fired power...
 rule: Continuous emissions monitoring requirements for compliance ...</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>rule: New Source Performance Standards for major industrial catego...
 rule: National Emission Standards for Hazardous Air Pollutants (NE...</t>
@@ -741,7 +741,7 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>rule: Civil penalties and consent decrees for violations (e.g., 20...</t>
         </is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>information: State Implementation Plans detailing how state will achieve ...
 information: Emissions inventories, air quality monitoring data, and comp...</t>
@@ -829,7 +829,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>money: Purchase of catalytic converters for all 1975+ model year ve...</t>
         </is>
@@ -864,7 +864,7 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>money: Purchase and installation of scrubbers, electrostatic precip...</t>
         </is>
@@ -898,7 +898,7 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>money: Investment in pollution control technology to meet NSPS stan...</t>
         </is>
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>information: Independent scientific review of NAAQS criteria documents an...</t>
         </is>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>information: Air quality research on health effects, emissions modeling, ...</t>
         </is>
@@ -1112,12 +1112,12 @@
           <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>information: Legislative advocacy for Clean Air Act passage and amendment...</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>rule: Advocacy for stringent NAAQS, petitions for new standards, a...</t>
         </is>
@@ -1145,12 +1145,12 @@
           <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>information: Lobbying for technology feasibility timelines and economic i...</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>information: Technical comments on proposed rules, compliance cost analys...</t>
         </is>
@@ -1257,17 +1257,17 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Environmental Justice Communities</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Industrial facilities disproportionately impact environmental justice communities through proximity and exposure patterns</t>
+          <t>Automobile manufacturers forced to adopt catalytic converter technology beginning 1975 model year</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
@@ -1277,21 +1277,21 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Pollution Control Equipment Industry</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Industrial facilities install control technology to comply with federal and state emissions limits</t>
+          <t>Automobile manufacturers emit air pollutants that impact public health, with dramatic reductions post-1975 due to catalytic converters</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1302,32 +1302,32 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Justice Communities</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Industrial facilities emit criteria pollutants and hazardous air pollutants affecting nearby populations</t>
+          <t>Industrial facilities disproportionately impact environmental justice communities through proximity and exposure patterns</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Pollution Control Equipment Industry</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>DOJ enforces Clean Air Act through civil and criminal penalties against violators</t>
+          <t>Industrial facilities install control technology to comply with federal and state emissions limits</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
@@ -1337,37 +1337,37 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Technology suppliers provide emission control equipment enabling regulatory compliance</t>
+          <t>Industrial facilities emit criteria pollutants and hazardous air pollutants affecting nearby populations</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Air Quality Research Institutions</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Research institutions provide scientific basis for NAAQS and regulatory decisions</t>
+          <t>DOJ enforces Clean Air Act through civil and criminal penalties against violators</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
@@ -1377,57 +1377,57 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>EPA regulates electric power plant emissions through NSPS and SIP requirements</t>
+          <t>Industry trade groups advocate for flexible compliance timelines and cost considerations in rulemaking</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>EPA regulates industrial emissions through technology-based standards</t>
+          <t>Industry associations lobby Congress on compliance timelines and economic impacts</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>EPA refers significant violations to Department of Justice for enforcement actions</t>
+          <t>Technology suppliers provide emission control equipment enabling regulatory compliance</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
@@ -1442,16 +1442,16 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Clean Air Act implementation delivers substantial public health benefits through dramatic pollution reductions</t>
+          <t>EPA regulates electric power plant emissions through NSPS and SIP requirements</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1482,32 +1482,32 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>EPA sets national air quality standards that states must achieve through SIPs</t>
+          <t>EPA regulates industrial emissions through technology-based standards</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Industry trade groups advocate for flexible compliance timelines and cost considerations in rulemaking</t>
+          <t>EPA refers significant violations to Department of Justice for enforcement actions</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
@@ -1517,17 +1517,17 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Industry associations lobby Congress on compliance timelines and economic impacts</t>
+          <t>Clean Air Act implementation delivers substantial public health benefits through dramatic pollution reductions</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
@@ -1537,37 +1537,37 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CASAC provides independent scientific peer review of air quality standards since 1977</t>
+          <t>EPA sets national air quality standards that states must achieve through SIPs</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Automobile manufacturers forced to adopt catalytic converter technology beginning 1975 model year</t>
+          <t>CASAC provides independent scientific peer review of air quality standards since 1977</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
@@ -1577,47 +1577,47 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Automobile manufacturers emit air pollutants that impact public health, with dramatic reductions post-1975 due to catalytic converters</t>
+          <t>Environmental organizations advocate for strong air quality protections and sue to enforce compliance</t>
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>States submit implementation plans for EPA approval, demonstrating path to NAAQS compliance</t>
+          <t>Environmental groups mobilize public support and provide legislative advocacy for air quality laws</t>
         </is>
       </c>
       <c r="D21" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -1627,37 +1627,37 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Environmental organizations advocate for strong air quality protections and sue to enforce compliance</t>
+          <t>Congress grants EPA regulatory authority over air pollution through NAAQS, NSPS, NESHAPS, and mobile source standards</t>
         </is>
       </c>
       <c r="D22" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Environmental groups mobilize public support and provide legislative advocacy for air quality laws</t>
+          <t>Congress mandates state leadership in air quality management through State Implementation Plans</t>
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Air Quality Research Institutions</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1667,27 +1667,27 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Congress grants EPA regulatory authority over air pollution through NAAQS, NSPS, NESHAPS, and mobile source standards</t>
+          <t>Research institutions provide scientific basis for NAAQS and regulatory decisions</t>
         </is>
       </c>
       <c r="D24" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Congress mandates state leadership in air quality management through State Implementation Plans</t>
+          <t>States submit implementation plans for EPA approval, demonstrating path to NAAQS compliance</t>
         </is>
       </c>
       <c r="D25" s="10" t="n">
@@ -1884,27 +1884,37 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Environmental Justice Communities</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Disproportionate exposure to industrial air pollution in low-income and minority communities located near facilities</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
+          <t>Purchase of catalytic converters for all 1975+ model year vehicles at $300-1000 per unit</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>USD per vehicle</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H5" s="11" t="n"/>
       <c r="I5" s="11" t="n">
         <v>0.9</v>
@@ -1913,40 +1923,48 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Pollution Control Equipment Industry</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Investment in pollution control technology to meet NSPS standards</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="9" t="n"/>
+          <t>Nitrogen oxides from vehicles: 5.2 kg/km²/day (1970) reduced to 2.2 kg/km²/day by 2010</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>kg/km²/day</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>continuous</t>
         </is>
       </c>
-      <c r="H6" s="11" t="n"/>
+      <c r="H6" s="11" t="n">
+        <v>2.2</v>
+      </c>
       <c r="I6" s="11" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -1961,25 +1979,13 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Sulfur dioxide from industrial sources: 5.6 kg/km²/day (1970) reduced to 0.6 kg/km²/day by 2010</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>kg/km²/day</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>0.6</v>
-      </c>
+          <t>Particulate matter from vehicles: &gt;90% reduction from 1970 levels due to diesel particulate filters and cleaner engines</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="11" t="n"/>
       <c r="I7" s="11" t="n">
         <v>0.95</v>
       </c>
@@ -1992,7 +1998,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Justice Communities</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -2002,7 +2008,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Particulate matter from industry: 50% reduction by 1980 through industrial emission controls</t>
+          <t>Disproportionate exposure to industrial air pollution in low-income and minority communities located near facilities</t>
         </is>
       </c>
       <c r="E8" s="11" t="n"/>
@@ -2010,73 +2016,79 @@
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="11" t="n"/>
       <c r="I8" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Pollution Control Equipment Industry</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Civil penalties and consent decrees for violations (e.g., 2024 enforcement actions: $13M+ in penalties)</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>13000000</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>USD in penalties</t>
-        </is>
-      </c>
+          <t>Investment in pollution control technology to meet NSPS standards</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="9" t="n"/>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>event_triggered</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Catalytic converter technology enabling 90% reduction in hydrocarbons and CO emissions</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="11" t="n"/>
+          <t>Sulfur dioxide from industrial sources: 5.6 kg/km²/day (1970) reduced to 0.6 kg/km²/day by 2010</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>kg/km²/day</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>0.6</v>
+      </c>
       <c r="I10" s="11" t="n">
         <v>0.95</v>
       </c>
@@ -2084,45 +2096,41 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Air Quality Research Institutions</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>pollution</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Air quality research on health effects, emissions modeling, and control technology effectiveness</t>
+          <t>Particulate matter from industry: 50% reduction by 1980 through industrial emission controls</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G11" s="9" t="n"/>
       <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -2132,36 +2140,46 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>New Source Performance Standards (NSPS) for coal-fired power plants limiting SO2 and NOx emissions</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
+          <t>Civil penalties and consent decrees for violations (e.g., 2024 enforcement actions: $13M+ in penalties)</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>USD in penalties</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>event_triggered</t>
+        </is>
+      </c>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Electric Power Plants</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Continuous emissions monitoring requirements for compliance verification</t>
+          <t>Technical comments on proposed rules, compliance cost analyses, requests for deadline extensions</t>
         </is>
       </c>
       <c r="E13" s="11" t="n"/>
@@ -2173,28 +2191,28 @@
       </c>
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>New Source Performance Standards for major industrial categories (steel, cement, chemicals)</t>
+          <t>Lobbying for technology feasibility timelines and economic impact considerations in legislation</t>
         </is>
       </c>
       <c r="E14" s="11" t="n"/>
@@ -2202,28 +2220,28 @@
       <c r="G14" s="9" t="n"/>
       <c r="H14" s="11" t="n"/>
       <c r="I14" s="11" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>Catalytic Converter Manufacturers</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
+          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>National Emission Standards for Hazardous Air Pollutants (NESHAPS)</t>
+          <t>Catalytic converter technology enabling 90% reduction in hydrocarbons and CO emissions</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -2231,7 +2249,7 @@
       <c r="G15" s="9" t="n"/>
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="16">
@@ -2242,29 +2260,25 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Referrals of Clean Air Act violations for civil and criminal prosecution</t>
+          <t>New Source Performance Standards (NSPS) for coal-fired power plants limiting SO2 and NOx emissions</t>
         </is>
       </c>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G16" s="9" t="n"/>
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2275,25 +2289,29 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Electric Power Plants</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dramatic air quality improvements: PM2.5 reduced to 35.1% of 1970 levels, combined six pollutants down 78% (1970-2020)</t>
+          <t>Continuous emissions monitoring requirements for compliance verification</t>
         </is>
       </c>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="9" t="n"/>
-      <c r="G17" s="9" t="n"/>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2397,7 +2415,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -2407,7 +2425,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>National Ambient Air Quality Standards for six criteria pollutants (CO, lead, NO2, ozone, PM, SO2)</t>
+          <t>New Source Performance Standards for major industrial categories (steel, cement, chemicals)</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
@@ -2426,17 +2444,17 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Industrial Facilities (Steel, Chemical, Manufacturing)</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Technical guidance for SIP development, emissions inventories, and monitoring requirements</t>
+          <t>National Emission Standards for Hazardous Air Pollutants (NESHAPS)</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
@@ -2444,7 +2462,7 @@
       <c r="G22" s="9" t="n"/>
       <c r="H22" s="11" t="n"/>
       <c r="I22" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2455,79 +2473,79 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>SIP approval authority and enforcement backstop (EPA can impose Federal Implementation Plan if state fails)</t>
+          <t>Referrals of Clean Air Act violations for civil and criminal prosecution</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H23" s="11" t="n"/>
       <c r="I23" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>American Public (210 million in 1970)</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Technical comments on proposed rules, compliance cost analyses, requests for deadline extensions</t>
+          <t>Dramatic air quality improvements: PM2.5 reduced to 35.1% of 1970 levels, combined six pollutants down 78% (1970-2020)</t>
         </is>
       </c>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="9" t="n"/>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G24" s="9" t="n"/>
       <c r="H24" s="11" t="n"/>
       <c r="I24" s="11" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Industry Trade Associations (NAM, API, Motor Vehicle Manufacturers Assoc.)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Lobbying for technology feasibility timelines and economic impact considerations in legislation</t>
+          <t>National Ambient Air Quality Standards for six criteria pollutants (CO, lead, NO2, ozone, PM, SO2)</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -2535,18 +2553,18 @@
       <c r="G25" s="9" t="n"/>
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -2556,139 +2574,121 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Independent scientific review of NAAQS criteria documents and recommendations (established 1977 amendments)</t>
+          <t>Technical guidance for SIP development, emissions inventories, and monitoring requirements</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="9" t="n"/>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G26" s="9" t="n"/>
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="11" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Catalytic Converter Manufacturers</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Purchase of catalytic converters for all 1975+ model year vehicles at $300-1000 per unit</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="n">
-        <v>500</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>USD per vehicle</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+          <t>SIP approval authority and enforcement backstop (EPA can impose Federal Implementation Plan if state fails)</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="9" t="n"/>
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Clean Air Scientific Advisory Committee (CASAC)</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Nitrogen oxides from vehicles: 5.2 kg/km²/day (1970) reduced to 2.2 kg/km²/day by 2010</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>kg/km²/day</t>
-        </is>
-      </c>
+          <t>Independent scientific review of NAAQS criteria documents and recommendations (established 1977 amendments)</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="9" t="n"/>
       <c r="G28" s="9" t="inlineStr">
         <is>
           <t>continuous</t>
         </is>
       </c>
-      <c r="H28" s="11" t="n">
-        <v>2.2</v>
-      </c>
+      <c r="H28" s="11" t="n"/>
       <c r="I28" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Automobile Manufacturers (GM, Ford, Chrysler)</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>American Public (210 million in 1970)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>pollution</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Particulate matter from vehicles: &gt;90% reduction from 1970 levels due to diesel particulate filters and cleaner engines</t>
+          <t>Advocacy for stringent NAAQS, petitions for new standards, and litigation to enforce deadlines</t>
         </is>
       </c>
       <c r="E29" s="11" t="n"/>
       <c r="F29" s="9" t="n"/>
-      <c r="G29" s="9" t="n"/>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>State Implementation Plans detailing how state will achieve NAAQS (Utah submitted January 1972)</t>
+          <t>Legislative advocacy for Clean Air Act passage and amendments, public health documentation</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
@@ -2706,13 +2706,13 @@
       <c r="G30" s="9" t="n"/>
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -2722,30 +2722,26 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Emissions inventories, air quality monitoring data, and compliance reports</t>
+          <t>Legislative authority to set National Ambient Air Quality Standards (NAAQS) for six criteria pollutants</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+      <c r="G31" s="9" t="n"/>
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -2755,45 +2751,51 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Advocacy for stringent NAAQS, petitions for new standards, and litigation to enforce deadlines</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="9" t="n"/>
+          <t>Federal appropriations for EPA operations and grants to states</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="n">
+        <v>1400000000</v>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>USD/year</t>
+        </is>
+      </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>annual</t>
         </is>
       </c>
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Environmental Advocacy Organizations (NRDC, Sierra Club, EDF)</t>
+          <t>U.S. Congress</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Legislative advocacy for Clean Air Act passage and amendments, public health documentation</t>
+          <t>Mandatory deadlines: NAAQS by 1971, state compliance by 1975 (later extended to 1977)</t>
         </is>
       </c>
       <c r="E33" s="11" t="n"/>
@@ -2801,7 +2803,7 @@
       <c r="G33" s="9" t="n"/>
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="11" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2812,7 +2814,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -2822,7 +2824,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Legislative authority to set National Ambient Air Quality Standards (NAAQS) for six criteria pollutants</t>
+          <t>Requirement to develop State Implementation Plans (SIPs) to achieve NAAQS</t>
         </is>
       </c>
       <c r="E34" s="11" t="n"/>
@@ -2841,7 +2843,7 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Environmental Protection Agency (EPA)</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
@@ -2851,31 +2853,21 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Federal appropriations for EPA operations and grants to states</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>1400000000</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>USD/year</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>annual</t>
-        </is>
-      </c>
+          <t>Federal planning grants to state air pollution control agencies (authorized under 1967 Air Quality Act, continued)</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>Air Quality Research Institutions</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -2885,41 +2877,45 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Mandatory deadlines: NAAQS by 1971, state compliance by 1975 (later extended to 1977)</t>
+          <t>Air quality research on health effects, emissions modeling, and control technology effectiveness</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
       <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="11" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Requirement to develop State Implementation Plans (SIPs) to achieve NAAQS</t>
+          <t>State Implementation Plans detailing how state will achieve NAAQS (Utah submitted January 1972)</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -2933,30 +2929,34 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>U.S. Congress</t>
+          <t>State Air Pollution Control Agencies (50 states)</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>State Air Pollution Control Agencies (50 states)</t>
+          <t>Environmental Protection Agency (EPA)</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Federal planning grants to state air pollution control agencies (authorized under 1967 Air Quality Act, continued)</t>
+          <t>Emissions inventories, air quality monitoring data, and compliance reports</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
       <c r="F38" s="9" t="n"/>
-      <c r="G38" s="9" t="n"/>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>